<commit_message>
add question data about arteries and veins in the circulatory system and include level and hint columns.
</commit_message>
<xml_diff>
--- a/ai/data/raw/Project_CirculatorySystem_QDatas.xlsx
+++ b/ai/data/raw/Project_CirculatorySystem_QDatas.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="305">
   <si>
     <t>id</t>
   </si>
@@ -37,6 +37,9 @@
     <t>tags</t>
   </si>
   <si>
+    <t>level</t>
+  </si>
+  <si>
     <t>question_text</t>
   </si>
   <si>
@@ -46,6 +49,9 @@
     <t>answer</t>
   </si>
   <si>
+    <t>hint</t>
+  </si>
+  <si>
     <t>rationale</t>
   </si>
   <si>
@@ -73,6 +79,9 @@
     <t>heart; function; circulation</t>
   </si>
   <si>
+    <t>easy</t>
+  </si>
+  <si>
     <t>Kalp, kasılma ve gevşeme hareketleri ile kanın damarlar içinde dolaşmasını sağlayan bir pompa görevi görür.</t>
   </si>
   <si>
@@ -82,6 +91,9 @@
     <t>{"correct_index":0}</t>
   </si>
   <si>
+    <t>Kalbin dolaşım sistemindeki temel rolünü düşün.</t>
+  </si>
+  <si>
     <t>Ders kitabı s.131</t>
   </si>
   <si>
@@ -100,6 +112,9 @@
     <t>{"correct_index":1}</t>
   </si>
   <si>
+    <t>Kalbin göğüs boşluğundaki yerini hatırla.</t>
+  </si>
+  <si>
     <t>Ders kitabına göre, kalp mediastinumda yer alır ve büyük kısmı orta hattın solunda olsa da bir bölümü sağ tarafta bulunur.</t>
   </si>
   <si>
@@ -115,6 +130,9 @@
     <t>Sağ ventrikül kanı tüm vücuda pompalar.</t>
   </si>
   <si>
+    <t>Sağ ve sol ventrikülün kanı nereye pompaladığını hatırla.</t>
+  </si>
+  <si>
     <t>Ders kitabına göre, sağ ventrikül kanı akciğerlere gönderir, tüm vücuda pompalayan sol ventriküldür.</t>
   </si>
   <si>
@@ -130,6 +148,9 @@
     <t>Kalpteki septumlar, temiz ve kirli kanın birbirine karışmasını engeller.</t>
   </si>
   <si>
+    <t>Kalbin sağ ve sol tarafındaki kanın karışıp karışmadığını düşün.</t>
+  </si>
+  <si>
     <t>heart_wall_layers_tf_01</t>
   </si>
   <si>
@@ -139,9 +160,15 @@
     <t>heart; myocardium; heart wall; cardiac anatomy; heart layers</t>
   </si>
   <si>
+    <t>medium</t>
+  </si>
+  <si>
     <t>Kalp duvarının en kalın tabakası endokarddır.</t>
   </si>
   <si>
+    <t>Kalp duvarındaki kas tabakasının adını hatırla.</t>
+  </si>
+  <si>
     <t>Ders kitabına göre, kalp duvarının en kalın tabakası kas tabakası olan miyokarddır.</t>
   </si>
   <si>
@@ -157,6 +184,9 @@
     <t>Koroner arterler pulmoner arterden ayrılan ilk dallardır.</t>
   </si>
   <si>
+    <t>Koroner arterlerin hangi büyük damardan ayrıldığını düşün.</t>
+  </si>
+  <si>
     <t>Ders kitabına göre, koroner arterler aorttan ayrılan ilk dallardır.</t>
   </si>
   <si>
@@ -175,6 +205,9 @@
     <t>Kalpte bulunan dört kapağın ikisi atriyoventriküler, ikisi semilunar kapaktır.</t>
   </si>
   <si>
+    <t>Kalpteki kapakların türlerini ve sayısını hatırla.</t>
+  </si>
+  <si>
     <t>coronary_artery_tf_02</t>
   </si>
   <si>
@@ -187,6 +220,9 @@
     <t>Koroner sinüs, kalp kasından gelen kirli kanı toplayarak sağ atriyuma iletir.</t>
   </si>
   <si>
+    <t xml:space="preserve"> Koroner sinüsün kalpteki venöz kanı nereye taşıdığını düşün.</t>
+  </si>
+  <si>
     <t>Ders kitabına göre, koroner venler birleşerek koroner sinüsü oluşturur ve buradaki kan sağ atriyuma dökülür.</t>
   </si>
   <si>
@@ -202,6 +238,9 @@
     <t>Miyokard tabakası atriyumlarda ventriküllere göre daha kalındır.</t>
   </si>
   <si>
+    <t>Atriyum ve ventriküllerin pompalama gücünü karşılaştır.</t>
+  </si>
+  <si>
     <t>Ders kitabına göre,miyokard ventriküllerde, özellikle sol ventrikülde daha kalındır.</t>
   </si>
   <si>
@@ -226,6 +265,9 @@
     <t>{"correct_index":2}</t>
   </si>
   <si>
+    <t>Sistemik dolaşıma kan gönderen ventrikülü düşün.</t>
+  </si>
+  <si>
     <t>Ders kitabına göre, sol ventrikül oksijen bakımından zengin kanı aort aracılığıyla tüm vücuda pompalar.</t>
   </si>
   <si>
@@ -244,6 +286,9 @@
     <t>{"options":["Septum interatriale","Septum interventrikulare","Perikard","Endokard"]}</t>
   </si>
   <si>
+    <t xml:space="preserve"> Kalbin sağ ve sol ventriküllerini ayıran bölmeyi hatırla.</t>
+  </si>
+  <si>
     <t>Ders kitabına göre, septum interventrikulare sağ ve sol ventrikülü birbirinden ayırır.</t>
   </si>
   <si>
@@ -262,6 +307,9 @@
     <t>{"options":["Endokard","Miyokard","Perikard","Epikard"]}</t>
   </si>
   <si>
+    <t>Kalp duvarındaki kas tabakasını düşün.</t>
+  </si>
+  <si>
     <t>Ders kitabına göre, kalbin kasılmasını sağlayan tabaka miyokarddır ve ventriküllerde daha kalındır.</t>
   </si>
   <si>
@@ -274,12 +322,15 @@
     <t>heart; valve; mitral; cardiac anatomy</t>
   </si>
   <si>
-    <t>Mitral kapak aşağıdaki yapılar arasında bulunur?</t>
+    <t>Mitral kapak aşağıdaki hangi yapılar arasında bulunur?</t>
   </si>
   <si>
     <t>{"options":["Sağ atriyum – sağ ventrikül","Sol atriyum – sol ventrikül","Sağ ventrikül – pulmoner arter","Sol ventrikül – aort"]}</t>
   </si>
   <si>
+    <t>Sol atriyum ile sol ventrikül arasındaki kapağı hatırla.</t>
+  </si>
+  <si>
     <t>Ders kitabına göre, mitral kapak sol atriyum ile sol ventrikül arasında yer alan atriyoventriküler kapaktır.</t>
   </si>
   <si>
@@ -292,12 +343,18 @@
     <t>heart; coronary artery; heart vessels; circulation</t>
   </si>
   <si>
+    <t>hard</t>
+  </si>
+  <si>
     <t>Koroner arterler aşağıdaki damarlardan hangisinden ayrılır?</t>
   </si>
   <si>
     <t>{"options":["Pulmoner arter","Vena cava superior","Aort","Pulmoner ven"]}</t>
   </si>
   <si>
+    <t>Kalpten çıkan en büyük atardamarı düşün.</t>
+  </si>
+  <si>
     <t>Ders kitabına göre, koroner arterler aorttan ayrılan ilk dallardır ve kalp kasını besler.</t>
   </si>
   <si>
@@ -316,6 +373,9 @@
     <t>{"options":["Akciğerlere kan taşımak","Kalp kasından gelen kirli kanı toplamak","Oksijenli kanı sol ventriküle iletmek","Atriyumların kasılmasını başlatmak"]}</t>
   </si>
   <si>
+    <t>Kalp kasından dönen kanın toplandığı yapıyı düşün.</t>
+  </si>
+  <si>
     <t>Ders kitabına göre,  koroner venler birleşerek koroner sinüsü oluşturur ve kan sağ atriyuma dökülür.</t>
   </si>
   <si>
@@ -334,6 +394,9 @@
     <t>{"options":["Mitral kapak","Triküspit kapak","Aort kapağı","Biküspit kapak"]}</t>
   </si>
   <si>
+    <t>Büyük damarlara açılan kapakları hatırla.</t>
+  </si>
+  <si>
     <t>Ders kitabına göre, aort ve pulmoner kapaklar semilunar kapak grubuna girer.</t>
   </si>
   <si>
@@ -346,7 +409,7 @@
     <t>heart; myocardium; ventricle; cardiac muscle</t>
   </si>
   <si>
-    <t xml:space="preserve"> Miyokardın en kalın olduğu kalp odacığı hangisidir?</t>
+    <t>Miyokardın en kalın olduğu kalp odacığı hangisidir?</t>
   </si>
   <si>
     <t>{"options":["Sağ atriyum","Sol atriyum","Sağ ventrikül","Sol ventrikül"]}</t>
@@ -355,6 +418,9 @@
     <t>{"correct_index":3}</t>
   </si>
   <si>
+    <t>En güçlü pompalama yapan odacığı düşün.</t>
+  </si>
+  <si>
     <t>Ders kitabına göre, sol ventrikül tüm vücuda kan pompaladığı için en kalın miyokard tabakasına sahiptir.</t>
   </si>
   <si>
@@ -373,6 +439,9 @@
     <t>{"options":["Mitral kapak","Triküspit kapak","Aort kapağı","Hiçbiri"]}</t>
   </si>
   <si>
+    <t>Kanın ventriküllerden büyük damarlara çıktığı kapakları düşün.</t>
+  </si>
+  <si>
     <t>Ders kitabına göre, sistol sırasında ventriküller kasılır, atriyoventriküler kapaklar kapanır ve semilunar kapaklar (aort ve pulmoner kapak) açılarak kanın atardamarlara pompalanmasını sağlar.</t>
   </si>
   <si>
@@ -419,6 +488,444 @@
   </si>
   <si>
     <t>Ders kitabı s.133</t>
+  </si>
+  <si>
+    <t>artery_wall_layers_tf_01</t>
+  </si>
+  <si>
+    <t>Atardamar duvarı - T/F</t>
+  </si>
+  <si>
+    <t>Vessels</t>
+  </si>
+  <si>
+    <t>artery; circulatory system; vessel structure; artery wall; tunica intima; tunica media; tunica adventitia; histology</t>
+  </si>
+  <si>
+    <t>Atardamar duvarı üç tabakadan oluşur: tunica intima, tunica media ve tunica adventitia.</t>
+  </si>
+  <si>
+    <t>Atardamarların histolojik katmanlarını düşün.</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.136</t>
+  </si>
+  <si>
+    <t>pulmonary_artery_tf_01</t>
+  </si>
+  <si>
+    <t>Akciğer atardamarı - T/F</t>
+  </si>
+  <si>
+    <t>artery; pulmonary circulation; pulmonary artery; arteria pulmonalis; right ventricle; lung circulation</t>
+  </si>
+  <si>
+    <t>Arteria pulmonalis kirli kanı akciğerlere taşır.</t>
+  </si>
+  <si>
+    <t>Sağ ventrikülden çıkan damarı düşün.</t>
+  </si>
+  <si>
+    <t>artery_tf_01</t>
+  </si>
+  <si>
+    <t>Atardamar basıncı - T/F</t>
+  </si>
+  <si>
+    <t>artery; blood pressure; arterial pressure; circulatory physiology; blood flow dynamics; vessel function</t>
+  </si>
+  <si>
+    <t>Atardamarlarda kan basıncı venlere göre daha düşüktür.</t>
+  </si>
+  <si>
+    <t>Kan kalpten hangi damarlara pompalanır?</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, atardamarlarda basınç venlere göre daha yüksektir çünkü kan doğrudan kalpten pompalanır.</t>
+  </si>
+  <si>
+    <t>aort_tf_01</t>
+  </si>
+  <si>
+    <t>Aort kemeri dalları - T/F</t>
+  </si>
+  <si>
+    <t>artery; aorta; aortic arch; truncus brachiocephalicus; systemic circulation; thoracic arteries</t>
+  </si>
+  <si>
+    <t>Aort kemerinden çıkan arterlerden biri truncus brachiocephalicus'tur.</t>
+  </si>
+  <si>
+    <t>Aort kemerinin ilk dalını düşün.</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.137</t>
+  </si>
+  <si>
+    <t>capillary_structure_tf_01</t>
+  </si>
+  <si>
+    <t>Kılcal damar yapısı - T/F</t>
+  </si>
+  <si>
+    <t>capillary; microcirculation; capillary wall; endothelial cells; diffusion; tissue exchange</t>
+  </si>
+  <si>
+    <t>Kılcal damarların duvarı tek katlı endotelden oluşur ve bu yapı madde alışverişini kolaylaştırır.</t>
+  </si>
+  <si>
+    <t>Gaz ve besin değişimi hangi damarlarda olur?</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.142</t>
+  </si>
+  <si>
+    <t>ertebral_basilar_tf_01</t>
+  </si>
+  <si>
+    <t>Vertebral arter birleşmesi - T/F</t>
+  </si>
+  <si>
+    <t>artery; vertebral artery; basilar artery; cerebral circulation; brain blood supply; willis polygon</t>
+  </si>
+  <si>
+    <t>Sağ ve sol vertebral arter birleşerek arteria carotis communis'i oluşturur.</t>
+  </si>
+  <si>
+    <t>Vertebral arterler hangi arteri oluşturur?</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, sağ ve sol vertebral arter birleşerek arteria basilaris'i oluşturur. Carotis communis ile ilişkili değildir.</t>
+  </si>
+  <si>
+    <t>artery_mcq_01</t>
+  </si>
+  <si>
+    <t>Atardamarlar - Görevi</t>
+  </si>
+  <si>
+    <t>artery; vessel function; systemic circulation; blood transport</t>
+  </si>
+  <si>
+    <t>Atardamarların temel görevi nedir?</t>
+  </si>
+  <si>
+    <t>{"options":["Kanı kalpten dokulara taşımak","Kanı dokulardan kalbe taşımak","Gaz değişimini sağlamak","Lenf sıvısını taşımak"]}</t>
+  </si>
+  <si>
+    <t>Kan kalpten hangi damarlarla çıkar?</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, atardamarlar kanı kalpten dokulara taşıyan damarlardır.</t>
+  </si>
+  <si>
+    <t>pulmonary_artery_mcq_01</t>
+  </si>
+  <si>
+    <t>Akciğer atardamarı</t>
+  </si>
+  <si>
+    <t>artery; pulmonary artery; right ventricle; lung circulation</t>
+  </si>
+  <si>
+    <t>Akciğer atardamarı hangi kalp boşluğundan çıkar?</t>
+  </si>
+  <si>
+    <t>{"options":["Sol atrium","Sol ventrikül","Sağ atrium","Sağ ventrikül"]}</t>
+  </si>
+  <si>
+    <t>Kirli kanın akciğere gittiği odayı hatırla</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, pulmoner arter sağ ventrikülden çıkar ve kirli kanı akciğerlere taşır.</t>
+  </si>
+  <si>
+    <t>capillary_structure_mcq_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kılcal damar - Yapısı  </t>
+  </si>
+  <si>
+    <t>capillary; microcirculation; vessel wall; endothelial cells</t>
+  </si>
+  <si>
+    <t>Kılcal damarların duvar yapısı nasıldır?</t>
+  </si>
+  <si>
+    <t>{"options":["Üç katlı kaslı yapı","İki katlı kaslı yapı","Tek katlı endotel","Kıkırdak doku"]}</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Madde alışverişi için ince yapı gerekir</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, kılcal damarların duvarı tek katlı endotelden oluşur.</t>
+  </si>
+  <si>
+    <t>aort_mcq_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aort kemeri - Dalları </t>
+  </si>
+  <si>
+    <t xml:space="preserve">artery; aorta; aortic arch; truncus brachiocephalicus </t>
+  </si>
+  <si>
+    <t>Aort kemerinden çıkan ilk dal aşağıdakilerden hangisidir?</t>
+  </si>
+  <si>
+    <t>{"options":["A. carotis communis sinistra","Truncus brachiocephalicus","A. subclavia sinistra","A. vertebralis"]}</t>
+  </si>
+  <si>
+    <t>Sağ baş ve kola giden arter buradan çıkar</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, aort kemerinin ilk dalı truncus brachiocephalicus'tur.</t>
+  </si>
+  <si>
+    <t>vertebral_artery_mcq_01</t>
+  </si>
+  <si>
+    <t>Vertebral arter</t>
+  </si>
+  <si>
+    <t>artery; vertebral artery; brain circulation; willis polygon</t>
+  </si>
+  <si>
+    <t>Vertebral arterlerin birleşmesiyle aşağıdaki damarlardan hangisi oluşur?</t>
+  </si>
+  <si>
+    <t>{"options":["A. carotis communis","A. basilaris","A. subclavia","A. axillaris"]}</t>
+  </si>
+  <si>
+    <t>Beynin tabanındaki arter</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, sağ ve sol vertebral arter birleşerek arteria basilaris'i oluşturur.</t>
+  </si>
+  <si>
+    <t>axillary_artery_mcq_01</t>
+  </si>
+  <si>
+    <t>A. axillaris - Konumu</t>
+  </si>
+  <si>
+    <t>artery; axillary artery; upper extremity; shoulder region</t>
+  </si>
+  <si>
+    <t>A. axillaris aşağıdaki bölgelerden hangisinde bulunur?</t>
+  </si>
+  <si>
+    <t>{"options":["Dirsek","Koltuk altı","Bilek","Boyun"]}</t>
+  </si>
+  <si>
+    <t>Subclavian arterin devamı olduğunu hatırla.</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, A. axillaris koltuk altı bölgesinde bulunur.</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.138</t>
+  </si>
+  <si>
+    <t>femoral_artery_mcq_01</t>
+  </si>
+  <si>
+    <t>Femoral arter - Konumu</t>
+  </si>
+  <si>
+    <t>artery; femoral artery; lower extremity; thigh circulation</t>
+  </si>
+  <si>
+    <t>A. femoralis hangi bölgede bulunur?</t>
+  </si>
+  <si>
+    <t>{"options":["Boyun","Uyluk","El bileği","Göğüs"]}</t>
+  </si>
+  <si>
+    <t>Latince femur kemiğini düşün.</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, femoral arter uyluk bölgesinde bulunur.</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.139</t>
+  </si>
+  <si>
+    <t>basilic_vein_mcq_01</t>
+  </si>
+  <si>
+    <t>V. basilica</t>
+  </si>
+  <si>
+    <t>vein; basilic vein; superficial veins; upper extremity</t>
+  </si>
+  <si>
+    <t>V. basilica hangi damar grubuna aittir?</t>
+  </si>
+  <si>
+    <t>{"options":["Derin arter","Yüzeyel ven","Lenf damarı","Kılcal damar"]}</t>
+  </si>
+  <si>
+    <t>Deri altında seyreden venleri hatırla.</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, V. basilica üst ekstremitenin yüzeyel venlerinden biridir.</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.140</t>
+  </si>
+  <si>
+    <t>vena_cava_mcq_01</t>
+  </si>
+  <si>
+    <t>Vena cava inferior oluşumu</t>
+  </si>
+  <si>
+    <t>vein; vena cava inferior; venous return; iliac veins; systemic circulation; toplardamar</t>
+  </si>
+  <si>
+    <t>Vena cava inferior aşağıdaki venlerden hangilerinin birleşmesi ile oluşur?</t>
+  </si>
+  <si>
+    <t>{"options":["Sağ ve sol V. iliaca communis","V. iliaca interna ve V. iliaca externa","V. femoralis ve V. poplitea","V. saphena magna ve V. saphena parva"]}</t>
+  </si>
+  <si>
+    <t>Alt ekstremiteden gelen büyük venlerin birleşmesini hatırla.</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, vena cava inferior, sağ ve sol vena iliaca communis venlerinin birleşmesiyle oluşur ve alt vücut bölgelerinden gelen venöz kanı kalbe taşır.</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.141</t>
+  </si>
+  <si>
+    <t>aort_mcq_02</t>
+  </si>
+  <si>
+    <t>İnen aort</t>
+  </si>
+  <si>
+    <t>artery; descending aorta; thoracic aorta; abdominal aorta</t>
+  </si>
+  <si>
+    <t>İnen aort aşağıdaki hangi iki bölümden oluşur?</t>
+  </si>
+  <si>
+    <t>{"options":["Torasik aort ve abdominal aort","Karotis ve vertebral arter","Aort kemeri ve aort kökü","Pulmoner arter ve pulmoner ven"]}</t>
+  </si>
+  <si>
+    <t>Göğüs ve karın bölgesini hatırla</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, inen aort göğüs aortu ve karın aortu olmak üzere iki bölüme ayrılır.</t>
+  </si>
+  <si>
+    <t>venous_mcq_01</t>
+  </si>
+  <si>
+    <t>Toplardamarların görevi</t>
+  </si>
+  <si>
+    <t>vein; venous return; systemic circulation; vena cava</t>
+  </si>
+  <si>
+    <t>Aşağıdakilerden hangisi toplardamarların temel özelliğidir?</t>
+  </si>
+  <si>
+    <t>{"options":["Kanı kalpten dokulara taşımaları","Yalnızca temiz kan taşımaları","Kanı dokulardan kalbe taşımaları","Yalnızca akciğerlerde bulunmaları"]}</t>
+  </si>
+  <si>
+    <t>Kanın dönüş yönünü düşün.</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, toplardamarlar kanı dokulardan kalbe geri taşıyan damarlardır.</t>
+  </si>
+  <si>
+    <t>pulse_artery_mcq_01</t>
+  </si>
+  <si>
+    <t>Nabız ölçümü</t>
+  </si>
+  <si>
+    <t>artery; radial artery; pulse measurement; clinical anatomy</t>
+  </si>
+  <si>
+    <t>Klinik muayenelerde nabız en sık hangi arterden ölçülür?</t>
+  </si>
+  <si>
+    <t>{"options":["A. axillaris","A. radialis","A. femoralis","A. subclavia"]}</t>
+  </si>
+  <si>
+    <t>Bilek bölgesini düşün</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, nabız ölçümü klinikte en sık radial arter üzerinden yapılır.</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.143</t>
+  </si>
+  <si>
+    <t>venous_return_order_mcq_01</t>
+  </si>
+  <si>
+    <t>Alt ekstremiteden venöz dönüş</t>
+  </si>
+  <si>
+    <t>vein; venous return; lower extremity veins; femoral vein; popliteal vein; iliac veins; vena cava inferior; toplardamar</t>
+  </si>
+  <si>
+    <t>Ayaktan kalbe doğru venöz kanın izlediği doğru sıra aşağıdakilerden hangisidir?</t>
+  </si>
+  <si>
+    <t>{"options":["V. tibialis posterior → V. poplitea → V. femoralis → V. iliaca externa → V. iliaca communis → V. cava inferior", "V. tibialis posterior → V. femoralis → V. poplitea → V. iliaca externa → V. cava inferior", "V. tibialis posterior → V. poplitea → V. iliaca communis → V. femoralis → V. cava inferior", "V. tibialis posterior → V. femoralis → V. iliaca externa → V. poplitea → V. cava inferior"]}</t>
+  </si>
+  <si>
+    <t>Diz arkasındaki venin adını hatırla.</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, alt ekstremitede venöz dönüş sırası tibialis venlerinden popliteaya, ardından femoral vene, sonra iliaca externa ve iliaca communis üzerinden vena cava inferiora ulaşır.</t>
+  </si>
+  <si>
+    <t>vessel_matching_01</t>
+  </si>
+  <si>
+    <t>Damarların Türkçe ve Latince karşılıkları</t>
+  </si>
+  <si>
+    <t>artery; vein; vessel terminology; latin names; anatomy</t>
+  </si>
+  <si>
+    <t>Aşağıdaki damarların Türkçe adları ile Latince karşılıklarını eşleştiriniz.</t>
+  </si>
+  <si>
+    <t>{"left":["Akciğer atardamarı", "Kol baş atardamarı", "Boyun iç toplardamarı", "Kapı toplardamarı"], "right":["Vena porta", "Arteria pulmonalis", "Vena jugularis interna", "Truncus brachiocephalicus"], "shuffle_right": true}</t>
+  </si>
+  <si>
+    <t>"pairs":[[0,1],[1,3],[2,2],[3,0]]</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.144</t>
+  </si>
+  <si>
+    <t>artery_body_region_matching_01</t>
+  </si>
+  <si>
+    <t>Arterler ve bulundukları bölgeler</t>
+  </si>
+  <si>
+    <t>artery; anatomical regions; systemic circulation; vessel location</t>
+  </si>
+  <si>
+    <t>Aşağıdaki arterleri bulundukları anatomik bölgeler ile eşleştiriniz.</t>
+  </si>
+  <si>
+    <t>{"left":["A. carotis communis", "A. axillaris", "A. brachialis", "A. femoralis", "A. poplitea", "A. dorsalis pedis"], "right":["Boyun","Koltuk altı","Kol","Uyluk","Diz arkası","Ayak sırtı"], "shuffle_right": true}</t>
+  </si>
+  <si>
+    <t>"pairs":[[0,0],[1,1],[2,2],[3,3],[4,4],[5,5]]</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.138–139</t>
   </si>
 </sst>
 </file>
@@ -708,7 +1215,7 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
@@ -720,807 +1227,1888 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E2" s="2">
         <v>30.0</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E3" s="2">
-        <v>30.0</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3" s="2" t="s">
+      <c r="L3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="O3" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E4" s="2">
         <v>30.0</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>34</v>
-      </c>
       <c r="M4" s="2" t="s">
-        <v>23</v>
+        <v>39</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="E5" s="2">
         <v>30.0</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>23</v>
+        <v>45</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="E6" s="2">
         <v>30.0</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>23</v>
+        <v>51</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="E7" s="2">
         <v>30.0</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>21</v>
+        <v>56</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>49</v>
+        <v>57</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="O7" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="E8" s="2">
         <v>30.0</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>53</v>
+        <v>22</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>21</v>
+        <v>63</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>49</v>
+        <v>64</v>
+      </c>
+      <c r="O8" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="E9" s="2">
         <v>30.0</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>57</v>
+        <v>22</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>21</v>
+        <v>68</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>49</v>
+        <v>69</v>
+      </c>
+      <c r="N9" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="O9" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="E10" s="2">
         <v>30.0</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>21</v>
+        <v>74</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>23</v>
+        <v>75</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="O10" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E11" s="2">
         <v>30.0</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>23</v>
+        <v>84</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="O11" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="E12" s="2">
         <v>30.0</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>75</v>
+        <v>49</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>28</v>
+        <v>90</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>77</v>
+        <v>32</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>23</v>
+        <v>91</v>
+      </c>
+      <c r="N12" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="O12" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>65</v>
-      </c>
       <c r="D13" s="2" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="E13" s="2">
         <v>30.0</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>81</v>
+        <v>49</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>83</v>
+        <v>32</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>23</v>
+        <v>98</v>
+      </c>
+      <c r="N13" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="O13" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="E14" s="2">
         <v>30.0</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>87</v>
+        <v>49</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>89</v>
+        <v>32</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>49</v>
+        <v>105</v>
+      </c>
+      <c r="N14" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="O14" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="E15" s="2">
         <v>30.0</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>94</v>
+        <v>111</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>70</v>
+        <v>112</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>49</v>
+        <v>113</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="O15" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>96</v>
+        <v>115</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>97</v>
+        <v>116</v>
       </c>
       <c r="E16" s="2">
         <v>30.0</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>99</v>
+        <v>49</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>100</v>
+        <v>118</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>28</v>
+        <v>119</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>101</v>
+        <v>32</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>49</v>
+        <v>120</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="O16" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>102</v>
+        <v>122</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>103</v>
+        <v>123</v>
       </c>
       <c r="E17" s="2">
         <v>30.0</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>104</v>
+        <v>124</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>105</v>
+        <v>49</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>106</v>
+        <v>125</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>70</v>
+        <v>126</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>107</v>
+        <v>83</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>49</v>
+        <v>127</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="O17" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>109</v>
+        <v>130</v>
       </c>
       <c r="E18" s="2">
         <v>30.0</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H18" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="I18" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="I18" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="J18" s="2" t="s">
-        <v>112</v>
+        <v>132</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>113</v>
+        <v>133</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>114</v>
+        <v>134</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>49</v>
+        <v>135</v>
+      </c>
+      <c r="N18" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="O18" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>116</v>
+        <v>138</v>
       </c>
       <c r="E19" s="2">
         <v>30.0</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>119</v>
+        <v>140</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>70</v>
+        <v>141</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>120</v>
+        <v>83</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>121</v>
+        <v>142</v>
+      </c>
+      <c r="N19" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="O19" s="2" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>122</v>
+        <v>145</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>123</v>
+        <v>146</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>124</v>
+        <v>147</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>125</v>
+        <v>148</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>126</v>
+        <v>49</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>127</v>
+        <v>149</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="M20" s="2" t="s">
-        <v>49</v>
+        <v>150</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="M20" s="2"/>
+      <c r="O20" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>129</v>
+        <v>152</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>123</v>
+        <v>146</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>130</v>
+        <v>153</v>
       </c>
       <c r="F21" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="M21" s="2"/>
+      <c r="O21" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G21" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="J21" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="K21" s="2" t="s">
+      <c r="D22" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="E22" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="O22" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="E23" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L23" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M23" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="O23" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="E24" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L24" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M24" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="N24" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="O24" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E25" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L25" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M25" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="O25" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="E26" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L26" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M26" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="O26" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="E27" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L27" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M27" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="N27" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="O27" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="E28" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="L28" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M28" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="N28" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="O28" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="E29" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="L29" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="M21" s="2" t="s">
-        <v>135</v>
+      <c r="M29" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="N29" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="O29" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E30" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="L30" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="M30" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="N30" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="O30" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="E31" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="L31" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M31" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="N31" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="O31" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="E32" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="L32" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M32" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="N32" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="O32" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="E33" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="K33" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="L33" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M33" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="N33" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="O33" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="E34" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="L34" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M34" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="N34" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="O34" s="2" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="E35" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J35" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="K35" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="L35" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M35" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="N35" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="O35" s="2" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="E36" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M36" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="N36" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="O36" s="2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="E37" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="L37" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M37" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="N37" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="O37" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="E38" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="L38" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="M38" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="N38" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="O38" s="2" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="E39" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="L39" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M39" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="N39" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="O39" s="2" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="E40" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M40" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="N40" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="O40" s="2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="L41" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="O41" s="2" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="O42" s="2" t="s">
+        <v>304</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add systemic and pulmonary circulation question data
</commit_message>
<xml_diff>
--- a/ai/data/raw/Project_CirculatorySystem_QDatas.xlsx
+++ b/ai/data/raw/Project_CirculatorySystem_QDatas.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="436">
   <si>
     <t>id</t>
   </si>
@@ -85,7 +85,7 @@
     <t>Kalp, kasılma ve gevşeme hareketleri ile kanın damarlar içinde dolaşmasını sağlayan bir pompa görevi görür.</t>
   </si>
   <si>
-    <t>{"options":["True","False"]}</t>
+    <t>{"options":["Doğru","Yanlış"]}</t>
   </si>
   <si>
     <t>{"correct_index":0}</t>
@@ -217,10 +217,10 @@
     <t>heart; coronary sinus; cardiac veins; heart vessels; circulation</t>
   </si>
   <si>
-    <t>Koroner sinüs, kalp kasından gelen kirli kanı toplayarak sağ atriyuma iletir.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Koroner sinüsün kalpteki venöz kanı nereye taşıdığını düşün.</t>
+    <t>Koroner sinüs, kalp kasından gelen venöz kanı sol atriyuma taşır.</t>
+  </si>
+  <si>
+    <t>Koroner sinüsün kalpteki venöz kanı nereye taşıdığını düşün.</t>
   </si>
   <si>
     <t>Ders kitabına göre, koroner venler birleşerek koroner sinüsü oluşturur ve buradaki kan sağ atriyuma dökülür.</t>
@@ -241,7 +241,7 @@
     <t>Atriyum ve ventriküllerin pompalama gücünü karşılaştır.</t>
   </si>
   <si>
-    <t>Ders kitabına göre,miyokard ventriküllerde, özellikle sol ventrikülde daha kalındır.</t>
+    <t>Ders kitabına göre, miyokard ventriküllerde, özellikle sol ventrikülde daha kalındır.</t>
   </si>
   <si>
     <t>heart_chambers_mcq_01</t>
@@ -286,7 +286,7 @@
     <t>{"options":["Septum interatriale","Septum interventrikulare","Perikard","Endokard"]}</t>
   </si>
   <si>
-    <t xml:space="preserve"> Kalbin sağ ve sol ventriküllerini ayıran bölmeyi hatırla.</t>
+    <t>Kalbin sağ ve sol ventriküllerini ayıran bölmeyi hatırla.</t>
   </si>
   <si>
     <t>Ders kitabına göre, septum interventrikulare sağ ve sol ventrikülü birbirinden ayırır.</t>
@@ -376,13 +376,13 @@
     <t>Kalp kasından dönen kanın toplandığı yapıyı düşün.</t>
   </si>
   <si>
-    <t>Ders kitabına göre,  koroner venler birleşerek koroner sinüsü oluşturur ve kan sağ atriyuma dökülür.</t>
+    <t>Ders kitabına göre, koroner venler birleşerek koroner sinüsü oluşturur ve kan sağ atriyuma dökülür.</t>
   </si>
   <si>
     <t>heart_valves_mcq_02</t>
   </si>
   <si>
-    <t>Kalp kapakları -  Türleri</t>
+    <t>Kalp kapakları - Türleri</t>
   </si>
   <si>
     <t>heart; valves; atrioventricular; semilunar</t>
@@ -391,7 +391,7 @@
     <t>Aşağıdaki kapaklardan hangisi semilunar kapak grubuna girer?</t>
   </si>
   <si>
-    <t>{"options":["Mitral kapak","Triküspit kapak","Aort kapağı","Biküspit kapak"]}</t>
+    <t>{"options":["Mitral kapak","Triküspit kapak","Aort kapağı","Koroner sinüs"]}</t>
   </si>
   <si>
     <t>Büyük damarlara açılan kapakları hatırla.</t>
@@ -400,7 +400,7 @@
     <t>Ders kitabına göre, aort ve pulmoner kapaklar semilunar kapak grubuna girer.</t>
   </si>
   <si>
-    <t xml:space="preserve"> myocardium_mcq_01</t>
+    <t>myocardium_mcq_01</t>
   </si>
   <si>
     <t>Miyokard - Kalınlığı</t>
@@ -433,16 +433,16 @@
     <t>heart; cardiac cycle; systole; diastole; heart valves</t>
   </si>
   <si>
-    <t>Ventriküllerin kasıldığı sistol evresinde aşağıdaki kapaklardan hangisi açık durumdadır?</t>
-  </si>
-  <si>
-    <t>{"options":["Mitral kapak","Triküspit kapak","Aort kapağı","Hiçbiri"]}</t>
+    <t>Sol ventrikülün sistol evresinde aşağıdaki kapaklardan hangisi açık durumdadır?</t>
+  </si>
+  <si>
+    <t>{"options":["Mitral kapak","Triküspit kapak","Aort kapağı","Pulmoner kapak"]}</t>
   </si>
   <si>
     <t>Kanın ventriküllerden büyük damarlara çıktığı kapakları düşün.</t>
   </si>
   <si>
-    <t>Ders kitabına göre, sistol sırasında ventriküller kasılır, atriyoventriküler kapaklar kapanır ve semilunar kapaklar (aort ve pulmoner kapak) açılarak kanın atardamarlara pompalanmasını sağlar.</t>
+    <t>Ders kitabına göre, sol ventrikül sistolünde ventrikül kasılır ve kan aort aracılığıyla sistemik dolaşıma gönderilir. Bu sırada aort kapağı açılır. Atriyoventriküler kapaklar (mitral ve triküspit kapak) ise kanın atriyumlara geri kaçmasını önlemek için kapalıdır.</t>
   </si>
   <si>
     <t>Ders kitabı s.134</t>
@@ -466,7 +466,7 @@
     <t>{"left":["Mitral kapak","Triküspit kapak","Aort kapağı","Pulmoner kapak"],"right":["Sağ ventrikül ile pulmoner arter arasında bulunur","Sol ventrikül ile aort arasında bulunur","Sağ atriyum ile sağ ventrikül arasında bulunur","Sol atriyum ile sol ventrikül arasında bulunur"],"shuffle_right":true}</t>
   </si>
   <si>
-    <t>{"pairs":[[0,3],[1,2],[2,1],[3,0]]}</t>
+    <t>{"pairs":[{"leftIndex":0,"rightIndex":3},{"leftIndex":1,"rightIndex":2},{"leftIndex":2,"rightIndex":1},{"leftIndex":3,"rightIndex":0}]}</t>
   </si>
   <si>
     <t>cardiac_conduction_system_matching_01</t>
@@ -484,7 +484,7 @@
     <t>{"left":["Sinoatriyal (SA) düğüm","Atriyoventriküler (AV) düğüm","His demeti","Purkinje lifleri"],"right":["Uyarıyı ventrikül kas tabakasına yayarak ventriküllerin kasılmasını sağlar","Kalpte ilk uyarının çıktığı merkezdir","Uyarıyı atriyumlardan ventriküllere kontrollü şekilde iletir","Uyarıyı ventriküller arası septum boyunca aşağı taşır"],"shuffle_right":true}</t>
   </si>
   <si>
-    <t>{"pairs":[[0,1],[1,2],[2,3],[3,0]]}</t>
+    <t>{"pairs":[{"leftIndex":0,"rightIndex":1},{"leftIndex":1,"rightIndex":2},{"leftIndex":2,"rightIndex":3},{"leftIndex":3,"rightIndex":0}]}</t>
   </si>
   <si>
     <t>Ders kitabı s.133</t>
@@ -580,7 +580,7 @@
     <t>Ders kitabı s.142</t>
   </si>
   <si>
-    <t>ertebral_basilar_tf_01</t>
+    <t>vertebral_basilar_tf_01</t>
   </si>
   <si>
     <t>Vertebral arter birleşmesi - T/F</t>
@@ -631,7 +631,7 @@
     <t>Akciğer atardamarı hangi kalp boşluğundan çıkar?</t>
   </si>
   <si>
-    <t>{"options":["Sol atrium","Sol ventrikül","Sağ atrium","Sağ ventrikül"]}</t>
+    <t>{"options":["Sol atriyum","Sol ventrikül","Sağ atriyum","Sağ ventrikül"]}</t>
   </si>
   <si>
     <t>Kirli kanın akciğere gittiği odayı hatırla</t>
@@ -643,7 +643,7 @@
     <t>capillary_structure_mcq_01</t>
   </si>
   <si>
-    <t xml:space="preserve">Kılcal damar - Yapısı  </t>
+    <t>Kılcal damar - Yapısı</t>
   </si>
   <si>
     <t>capillary; microcirculation; vessel wall; endothelial cells</t>
@@ -655,7 +655,7 @@
     <t>{"options":["Üç katlı kaslı yapı","İki katlı kaslı yapı","Tek katlı endotel","Kıkırdak doku"]}</t>
   </si>
   <si>
-    <t xml:space="preserve"> Madde alışverişi için ince yapı gerekir</t>
+    <t>Madde alışverişi için ince yapı gerekir</t>
   </si>
   <si>
     <t>Ders kitabına göre, kılcal damarların duvarı tek katlı endotelden oluşur.</t>
@@ -664,7 +664,7 @@
     <t>aort_mcq_01</t>
   </si>
   <si>
-    <t xml:space="preserve">Aort kemeri - Dalları </t>
+    <t>Aort kemeri - Dalları</t>
   </si>
   <si>
     <t xml:space="preserve">artery; aorta; aortic arch; truncus brachiocephalicus </t>
@@ -898,10 +898,10 @@
     <t>Aşağıdaki damarların Türkçe adları ile Latince karşılıklarını eşleştiriniz.</t>
   </si>
   <si>
-    <t>{"left":["Akciğer atardamarı", "Kol baş atardamarı", "Boyun iç toplardamarı", "Kapı toplardamarı"], "right":["Vena porta", "Arteria pulmonalis", "Vena jugularis interna", "Truncus brachiocephalicus"], "shuffle_right": true}</t>
-  </si>
-  <si>
-    <t>"pairs":[[0,1],[1,3],[2,2],[3,0]]</t>
+    <t>{"left":["Akciğer atardamarı", "Kol baş atardamarı", "Boyun iç toplardamarı", "Kapı toplardamarı"], "right":["Vena portae", "Arteria pulmonalis", "Vena jugularis interna", "Truncus brachiocephalicus"], "shuffle_right": true}</t>
+  </si>
+  <si>
+    <t>{"pairs":[{"leftIndex":0,"rightIndex":1},{"leftIndex":1,"rightIndex":3},{"leftIndex":2,"rightIndex":2},{"leftIndex":3,"rightIndex":0}]}</t>
   </si>
   <si>
     <t>Ders kitabı s.144</t>
@@ -922,10 +922,403 @@
     <t>{"left":["A. carotis communis", "A. axillaris", "A. brachialis", "A. femoralis", "A. poplitea", "A. dorsalis pedis"], "right":["Boyun","Koltuk altı","Kol","Uyluk","Diz arkası","Ayak sırtı"], "shuffle_right": true}</t>
   </si>
   <si>
-    <t>"pairs":[[0,0],[1,1],[2,2],[3,3],[4,4],[5,5]]</t>
+    <t>{"pairs":[{"leftIndex":0,"rightIndex":0},{"leftIndex":1,"rightIndex":1},{"leftIndex":2,"rightIndex":2},{"leftIndex":3,"rightIndex":3},{"leftIndex":4,"rightIndex":4},{"leftIndex":5,"rightIndex":5}]}</t>
   </si>
   <si>
     <t>Ders kitabı s.138–139</t>
+  </si>
+  <si>
+    <t>systemic_circulation_tf_01</t>
+  </si>
+  <si>
+    <t>Büyük kan dolaşımı - T/F</t>
+  </si>
+  <si>
+    <t>Circulation</t>
+  </si>
+  <si>
+    <t>circulation; systemic_circulation; oxygenated_blood; blood_flow; body_tissues; heart_pump; systemic_pathway</t>
+  </si>
+  <si>
+    <t>Büyük kan dolaşımı, oksijen bakımından zengin kanın kalpten tüm vücut dokularına gönderilmesini sağlar.</t>
+  </si>
+  <si>
+    <t>Temiz kanın kalpten dokulara gönderildiği dolaşımı düşün.</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.145</t>
+  </si>
+  <si>
+    <t>pulmonary_circulation_tf_01</t>
+  </si>
+  <si>
+    <t>Küçük kan dolaşımı - T/F</t>
+  </si>
+  <si>
+    <t>circulation; pulmonary_circulation; lungs; oxygen_exchange; right_ventricle; left_atrium; pulmonary_pathway</t>
+  </si>
+  <si>
+    <t>Küçük kan dolaşımında kan sağ ventrikülden çıkarak akciğerlere gider ve oksijenlenmiş olarak sol atriyuma döner.</t>
+  </si>
+  <si>
+    <t>Akciğer dolaşımında kanın hangi odacıktan çıktığını hatırla.</t>
+  </si>
+  <si>
+    <t>pulmonary_circulation_tf_02</t>
+  </si>
+  <si>
+    <t>Küçük kan dolaşımı gaz değişimi - T/F</t>
+  </si>
+  <si>
+    <t>circulation; pulmonary_circulation; gas_exchange; alveoli; lungs; oxygen_diffusion; respiratory_function</t>
+  </si>
+  <si>
+    <t>Küçük kan dolaşımında gaz değişimi kalpte gerçekleşir.</t>
+  </si>
+  <si>
+    <t>Gaz değişiminin gerçekleştiği organı düşün.</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, gaz değişimi akciğerlerdeki alveollerde gerçekleşir, kalpte gerçekleşmez.</t>
+  </si>
+  <si>
+    <t>portal_circulation_tf_01</t>
+  </si>
+  <si>
+    <t>Portal dolaşım - T/F</t>
+  </si>
+  <si>
+    <t>circulation; portal_circulation; liver; digestive_organs; hepatic_portal_system; venous_flow</t>
+  </si>
+  <si>
+    <t>Portal dolaşımda sindirim organlarından gelen kan doğrudan kalbe gider.</t>
+  </si>
+  <si>
+    <t>Portal dolaşımda kanın önce uğradığı organı düşün.</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, portal dolaşımda kan önce karaciğere taşınır, doğrudan kalbe gitmez.</t>
+  </si>
+  <si>
+    <t>systemic_circulation_tf_02</t>
+  </si>
+  <si>
+    <t>Dokularda gaz değişimi - T/F</t>
+  </si>
+  <si>
+    <t>circulation; systemic_circulation; tissue_exchange; oxygen_delivery; carbon_dioxide_transport; capillary_exchange</t>
+  </si>
+  <si>
+    <t>Büyük kan dolaşımında dokularda gaz değişimi gerçekleşir ve kan karbondioksit bakımından zengin hale gelir.</t>
+  </si>
+  <si>
+    <t>Hücrelerin oksijeni kullandığını hatırla.</t>
+  </si>
+  <si>
+    <t>heart_circulation_tf_01</t>
+  </si>
+  <si>
+    <t>Büyük ve küçük dolaşım ilişkisi - T/F</t>
+  </si>
+  <si>
+    <t>circulation; pulmonary_circulation; systemic_circulation; right_ventricle; left_atrium; oxygenation; blood_flow</t>
+  </si>
+  <si>
+    <t>Küçük kan dolaşımında oksijenlenen kan pulmoner venler aracılığıyla sağ atriyuma döner ve buradan büyük kan dolaşımı başlar.</t>
+  </si>
+  <si>
+    <t>Akciğerlerden gelen kanın hangi kalp odacığına döndüğünü hatırla.</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, akciğerlerde oksijenlenen kan pulmoner venler ile sol atriyuma döner. Sağ atriyuma dönmez.</t>
+  </si>
+  <si>
+    <t>systemic_circulation_mcq_01</t>
+  </si>
+  <si>
+    <t>Büyük kan dolaşımının başlangıcı</t>
+  </si>
+  <si>
+    <t>circulation; systemic_circulation; heart; left_ventricle; aorta; oxygenated_blood; blood_distribution; body_tissues</t>
+  </si>
+  <si>
+    <t>Büyük kan dolaşımında oksijen bakımından zengin kan aşağıdaki hangi kalp odacığından çıkar?</t>
+  </si>
+  <si>
+    <t>{"options":["Sol ventrikül","Sağ ventrikül","Sağ atriyum","Sol atriyum"]}</t>
+  </si>
+  <si>
+    <t>Aort hangi kalp odacığından çıkar?</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, büyük kan dolaşımında oksijenli kan sol ventrikülden aort aracılığıyla tüm vücuda gönderilir.</t>
+  </si>
+  <si>
+    <t>pulmonary_circulation_mcq_01</t>
+  </si>
+  <si>
+    <t>Küçük kan dolaşımı - Temel görevi</t>
+  </si>
+  <si>
+    <t>circulation; pulmonary_circulation; lungs; gas_exchange; oxygenation; respiratory_system; pulmonary_function</t>
+  </si>
+  <si>
+    <t>Küçük kan dolaşımının temel görevi aşağıdakilerden hangisidir?</t>
+  </si>
+  <si>
+    <t>{"options":["Kanın akciğerlerde oksijenlenmesini sağlamak","Kanın tüm vücuda dağıtılmasını sağlamak","Besin maddelerini karaciğere taşımak","Kanın kalbe geri dönmesini sağlamak"]}</t>
+  </si>
+  <si>
+    <t>Kanın temizlenmesi hangi organda gerçekleşir?</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, küçük dolaşım kirli kanı akciğerlere götürerek gaz değişimi ile oksijenlendirilmesini sağlar.</t>
+  </si>
+  <si>
+    <t>systemic_circulation_mcq_02</t>
+  </si>
+  <si>
+    <t>Büyük kan dolaşımı</t>
+  </si>
+  <si>
+    <t>circulation; systemic_circulation; tissue_exchange; oxygen_delivery; carbon_dioxide_transport; capillary_exchange; metabolism</t>
+  </si>
+  <si>
+    <t>Büyük kan dolaşımında dokularda gerçekleşen temel olay aşağıdakilerden hangisidir?</t>
+  </si>
+  <si>
+    <t>{"options":["Gaz değişimi gerçekleşmesi","Kanın kalbe pompalanması","Kanın akciğerlere gitmesi","Kapakların kapanması"]}</t>
+  </si>
+  <si>
+    <t>Bu olay kalpte veya akciğerde değil, vücut dokularında gerçekleşir.</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, dokularda oksijen hücreler tarafından kullanılır ve karbondioksit kana geçer.</t>
+  </si>
+  <si>
+    <t>pulmonary_circulation_mcq_02</t>
+  </si>
+  <si>
+    <t>Akciğerlerden kalbe dönen damar</t>
+  </si>
+  <si>
+    <t>circulation; pulmonary_circulation; pulmonary_vein; lungs; oxygenated_blood; heart_return; left_atrium</t>
+  </si>
+  <si>
+    <t>Küçük kan dolaşımında akciğerlerde oksijenlenen kan aşağıdaki damarlardan hangisi ile kalbe geri döner?</t>
+  </si>
+  <si>
+    <t>{"options":["Pulmoner ven","Pulmoner arter","Aort","Vena cava"]}</t>
+  </si>
+  <si>
+    <t>Akciğerlerden kalbe dönen damarları düşün.</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, akciğerlerde oksijenlenen kan pulmoner venlerle sol atriyuma döner.</t>
+  </si>
+  <si>
+    <t>pulmonary_circulation_mcq_03</t>
+  </si>
+  <si>
+    <t>Küçük dolaşımın başlangıç odacığı</t>
+  </si>
+  <si>
+    <t>circulation; pulmonary_circulation; right_ventricle; pulmonary_artery; lungs; blood_flow; pulmonary_pathway</t>
+  </si>
+  <si>
+    <t>Aşağıdakilerden hangisi küçük kan dolaşımının başlangıç noktasıdır?</t>
+  </si>
+  <si>
+    <t>{"options":["Sol ventrikül","Sağ ventrikül","Sol atriyum","Sağ atriyum"]}</t>
+  </si>
+  <si>
+    <t>Akciğerlere giden kan hangi ventrikülden çıkar?</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, küçük dolaşım sağ ventrikülden başlayan ve akciğerlere giden dolaşımdır.</t>
+  </si>
+  <si>
+    <t>systemic_circulation_mcq_03</t>
+  </si>
+  <si>
+    <t>Büyük kan dolaşımının sırası</t>
+  </si>
+  <si>
+    <t>circulation; systemic_circulation; blood_flow_pathway; heart_chambers; aorta; vena_cava</t>
+  </si>
+  <si>
+    <t>Aşağıdakilerden hangisi büyük kan dolaşımının doğru sırasını gösterir?</t>
+  </si>
+  <si>
+    <t>{"options":["Sol ventrikül → Aort → Vücut dokuları → Vena cava → Sağ atriyum","Sağ ventrikül → Aort → Akciğerler → Sol atriyum","Sol atriyum → Aort → Dokular → Sağ ventrikül","Sağ atriyum → Aort → Dokular → Sol atriyum"]}</t>
+  </si>
+  <si>
+    <t>Büyük dolaşımın kalbin sol tarafından başladığını hatırla.</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, büyük dolaşım sol ventrikül → aort → dokular → vena cava → sağ atriyum yolunu izler.</t>
+  </si>
+  <si>
+    <t>pulmonary_circulation_mcq_04</t>
+  </si>
+  <si>
+    <t>Küçük dolaşımda kanın izlediği yol</t>
+  </si>
+  <si>
+    <t>circulation; pulmonary_circulation; pulmonary_pathway; right_ventricle; pulmonary_artery; lungs</t>
+  </si>
+  <si>
+    <t>Küçük kan dolaşımında kanın izlediği doğru yol aşağıdakilerden hangisidir?</t>
+  </si>
+  <si>
+    <t>{"options":["Sol ventrikül → pulmoner arter → akciğer → pulmoner ven → sağ atriyum","Sağ atriyum → pulmoner arter → akciğer → vena cava → sol atriyum","Sol ventrikül → aort → akciğer → pulmoner ven → sağ atriyum","Sağ ventrikül → pulmoner arter → akciğer → pulmoner ven → sol atriyum"]}</t>
+  </si>
+  <si>
+    <t>Akciğerlere giden kanın çıktığı kalp odacığını düşün.</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, küçük kan dolaşımında kan sağ ventrikülden pulmoner arter ile akciğerlere gider, burada oksijenlenir ve pulmoner venler aracılığıyla sol atriyuma döner.</t>
+  </si>
+  <si>
+    <t>circulation_types_mcq_01</t>
+  </si>
+  <si>
+    <t>Büyük ve küçük dolaşım farkı</t>
+  </si>
+  <si>
+    <t>circulation; systemic_circulation; pulmonary_circulation; circulation_types; oxygen_transport; gas_exchange</t>
+  </si>
+  <si>
+    <t>Aşağıdakilerden hangisi büyük ve küçük kan dolaşımı arasındaki temel farklardan biridir?</t>
+  </si>
+  <si>
+    <t>{"options":["Büyük dolaşımda kan akciğerlere taşınırken küçük dolaşımda tüm vücut dokularına gönderilir","Küçük dolaşımda kan vena cava aracılığıyla kalbe dönerken büyük dolaşımda pulmoner venler kullanılır","Büyük dolaşım dokulara oksijen taşırken küçük dolaşım akciğerlerde gaz değişimini sağlar","Küçük dolaşım yalnızca kalp içinde gerçekleşen bir dolaşım yoludur"]}</t>
+  </si>
+  <si>
+    <t>Bir dolaşım vücut dokularıyla, diğeri akciğerlerle ilişkilidir.</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, büyük kan dolaşımı oksijen bakımından zengin kanı kalpten vücut dokularına taşır. Küçük kan dolaşımı ise kirli kanı akciğerlere götürerek gaz değişimini sağlar.</t>
+  </si>
+  <si>
+    <t>systemic_circulation_mcq_04</t>
+  </si>
+  <si>
+    <t>Büyük dolaşımda kanın kalbe dönüş yolu</t>
+  </si>
+  <si>
+    <t>circulation; systemic_circulation; venous_return; vena_cava; right_atrium; blood_flow; cardiovascular_system</t>
+  </si>
+  <si>
+    <t>Büyük kan dolaşımında vücut dokularında oksijenini kaybeden kanın kalbe dönüşünde aşağıdaki yapılardan hangisi son aşamayı oluşturur?</t>
+  </si>
+  <si>
+    <t>{"options":["Pulmoner arter","Aort","Vena cava","Pulmoner ven"]}</t>
+  </si>
+  <si>
+    <t>Vücuttan gelen kirli kanın kalbe döndüğü en büyük toplardamarı düşün.</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, vücut dokularında oksijenini kaybeden kan toplardamarlar aracılığıyla vena cava superior ve inferior üzerinden sağ atriyuma döner.</t>
+  </si>
+  <si>
+    <t>circulation_mcq_01</t>
+  </si>
+  <si>
+    <t>Dolaşım yolunda mantık hatası</t>
+  </si>
+  <si>
+    <t>circulation; pulmonary_circulation; systemic_circulation; blood_flow_pathway; heart_chambers</t>
+  </si>
+  <si>
+    <t>Bir öğrencinin kanın izlediği yolu şu şekilde tanımladığı düşünülüyor: “Vücut dokularında oksijenini kaybeden kan sağ atriyuma gelir, sağ ventriküle geçer ve akciğerlere gönderilir. Akciğerlerde oksijenlenen kan kalbe döndükten sonra sol ventriküle geçerek aort aracılığıyla tekrar vücuda gönderilir.” Bu açıklamada aşağıdaki hatalardan hangisi bulunmaktadır?</t>
+  </si>
+  <si>
+    <t>{"options":["Kirli kanın sağ atriyuma gelmesi yanlış ifade edilmiştir","Küçük dolaşımın sağ ventrikülden başlaması yanlış belirtilmiştir","Aortun büyük dolaşımda görev aldığı yanlış ifade edilmiştir","Akciğerlerden dönen kanın önce ulaştığı kalp odacığı eksik belirtilmiştir"]}</t>
+  </si>
+  <si>
+    <t>Akciğerlerden dönen kan kalpte hangi odacıktan geçerek sol ventriküle ulaşır?</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, akciğerlerde oksijenlenen kan pulmoner venler aracılığıyla önce sol atriyuma gelir, ardından sol ventriküle geçerek aort ile vücuda gönderilir. Öğrencinin açıklamasında sol atriyum basamağı atlanmıştır.</t>
+  </si>
+  <si>
+    <t>fetal_circulation_mcq_01</t>
+  </si>
+  <si>
+    <t>Foramen Ovale'nin görevi</t>
+  </si>
+  <si>
+    <t>circulation; fetal_circulation; foramen_ovale; fetal_heart; atrium; placental_circulation</t>
+  </si>
+  <si>
+    <t>Fetal dolaşımda foramen ovale yapısının temel görevi aşağıdakilerden hangisidir?</t>
+  </si>
+  <si>
+    <t>{"options":["Kanı pulmoner arterden aortaya yönlendirmek","Plasentadan gelen kanın karaciğere uğramadan vena cava inferiora geçmesini sağlamak","Sağ ve sol atriyum arasında kan geçişini sağlayarak akciğer dolaşımını büyük ölçüde atlamak","Vücut dokularından gelen kirli kanın plasentaya taşınmasını sağlamak"]}</t>
+  </si>
+  <si>
+    <t>Bu yapı fetüs kalbinde iki atriyum arasında bulunur.</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, foramen ovale, fetüste sağ ve sol atriyum arasında açıklık oluşturarak kanın doğrudan sol tarafa geçmesini sağlar. Böylece henüz çalışmayan akciğer dolaşımı büyük ölçüde bypass edilir.</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.146</t>
+  </si>
+  <si>
+    <t>lymph_circulation_mcq_01</t>
+  </si>
+  <si>
+    <t>Lenf sisteminde sıvı geri dönüşü</t>
+  </si>
+  <si>
+    <t>circulation; lymph_circulation; lymph_system; tissue_fluid; lymphatic_vessels; capillaries; lymph_return</t>
+  </si>
+  <si>
+    <t>Kılcal damarlarda gerçekleşen madde alışverişi sırasında dokulara geçen sıvının bir kısmı tekrar kana dönemez ve dokular arasında kalır. Bu sıvının dolaşım sistemine geri kazandırılmasını sağlayan yapı aşağıdakilerden hangisidir?</t>
+  </si>
+  <si>
+    <t>{"options":["Pulmoner arter","Aort","Lenf damarları","Koroner arterler"]}</t>
+  </si>
+  <si>
+    <t>Bu yapı doku sıvısını toplayarak tekrar dolaşıma kazandırır.</t>
+  </si>
+  <si>
+    <t>Ders kitabına göre, kılcal damarlarda dokulara geçen sıvının tamamı tekrar kana dönmez. Artan sıvı lenf kılcalları ve lenf damarları aracılığıyla toplanarak dolaşıma geri kazandırılır.</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.147</t>
+  </si>
+  <si>
+    <t>systemic_circulation_match_01</t>
+  </si>
+  <si>
+    <t>Büyük kan dolaşımının aşamaları</t>
+  </si>
+  <si>
+    <t>circulation; systemic_circulation; blood_flow; heart_chambers; aorta; vena_cava; circulation_pathway</t>
+  </si>
+  <si>
+    <t>Aşağıdaki yapıların büyük kan dolaşımındaki görevlerini eşleştiriniz.</t>
+  </si>
+  <si>
+    <t>{"left":["Sol ventrikül","Aort","Vücut dokuları","Vena cava"],"right":["Oksijen bakımından fakir kanı kalbe geri getirir","Oksijenli kanın vücuda pompalanmasını sağlar","Kanın tüm vücuda dağıldığı ana atardamardır","Doku hücreleri ile kan arasında madde alışverişi gerçekleşir"],"shuffle_right":true}</t>
+  </si>
+  <si>
+    <t>pulmonary_circulation_match_01</t>
+  </si>
+  <si>
+    <t>Küçük kan dolaşımının aşamaları</t>
+  </si>
+  <si>
+    <t>circulation; pulmonary_circulation; lungs; pulmonary_artery; pulmonary_vein; gas_exchange</t>
+  </si>
+  <si>
+    <t>Aşağıdaki yapıların küçük kan dolaşımındaki görevlerini eşleştiriniz.</t>
+  </si>
+  <si>
+    <t>{"left":["Sağ ventrikül","Pulmoner arter","Akciğer kılcal damarları","Pulmoner ven"],"right":["Oksijenlenmiş kanı kalbe taşır","Kirli kanı akciğerlere pompalar","Kirli kanı akciğerlere götüren damar","Gaz değişiminin gerçekleştiği damar ağı"],"shuffle_right":true}</t>
   </si>
 </sst>
 </file>
@@ -3111,6 +3504,922 @@
         <v>304</v>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="E43" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L43" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M43" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="O43" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E44" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L44" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M44" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="O44" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="E45" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J45" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L45" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M45" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="N45" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="O45" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="E46" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J46" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L46" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M46" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="N46" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="O46" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="E47" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J47" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L47" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M47" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="O47" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="E48" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="J48" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L48" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M48" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="N48" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="O48" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="E49" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J49" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="K49" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="L49" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M49" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="N49" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="O49" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="E50" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="K50" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="L50" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M50" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="N50" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="O50" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="E51" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J51" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="L51" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M51" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="N51" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="O51" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="E52" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="I52" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J52" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="L52" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M52" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="N52" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="O52" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="E53" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="I53" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J53" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="L53" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M53" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="N53" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="O53" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="E54" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J54" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="K54" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="L54" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M54" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="N54" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="O54" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E55" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J55" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="K55" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="L55" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="M55" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="N55" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="O55" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="E56" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="J56" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="L56" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="M56" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="N56" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="O56" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="E57" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="I57" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J57" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="K57" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="L57" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="M57" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="N57" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="O57" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="E58" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="J58" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="K58" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="L58" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="M58" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="N58" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="O58" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="E59" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="I59" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J59" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="K59" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="L59" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="M59" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="N59" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="O59" s="2" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E60" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="I60" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J60" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="K60" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="L60" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="M60" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="N60" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="O60" s="2" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="I61" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J61" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="K61" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="L61" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="O61" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H62" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="I62" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J62" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="K62" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="L62" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="O62" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="G63" s="2"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>